<commit_message>
json and 2 patient data implemented
</commit_message>
<xml_diff>
--- a/demoplay/src/test/resources/OPRegistrationDataJsonValidation.xlsx
+++ b/demoplay/src/test/resources/OPRegistrationDataJsonValidation.xlsx
@@ -25,6 +25,9 @@
     <t>PAY</t>
   </si>
   <si>
+    <t>FREE</t>
+  </si>
+  <si>
     <t>PatientType</t>
   </si>
   <si>
@@ -52,6 +55,9 @@
     <t>25-06-2001</t>
   </si>
   <si>
+    <t>25-06-2002</t>
+  </si>
+  <si>
     <t>Gender</t>
   </si>
   <si>
@@ -88,6 +94,9 @@
     <t>98 rrr street</t>
   </si>
   <si>
+    <t>99 rrr street</t>
+  </si>
+  <si>
     <t>locality</t>
   </si>
   <si>
@@ -145,7 +154,7 @@
     <t>PatientSubCategory</t>
   </si>
   <si>
-    <t>Subsidy</t>
+    <t>Concession</t>
   </si>
   <si>
     <t>SubsidyApprovedBy</t>
@@ -187,6 +196,9 @@
     <t>458967</t>
   </si>
   <si>
+    <t>458968</t>
+  </si>
+  <si>
     <t>Employee grade</t>
   </si>
   <si>
@@ -199,12 +211,18 @@
     <t>1526349</t>
   </si>
   <si>
+    <t>1523445</t>
+  </si>
+  <si>
     <t>Claim id</t>
   </si>
   <si>
     <t>1452</t>
   </si>
   <si>
+    <t>3048342</t>
+  </si>
+  <si>
     <t>Corporate remarks</t>
   </si>
   <si>
@@ -217,16 +235,22 @@
     <t>12563</t>
   </si>
   <si>
+    <t>12564</t>
+  </si>
+  <si>
     <t>Reference date</t>
   </si>
   <si>
     <t>20-06-2026</t>
   </si>
   <si>
+    <t>20-06-2027</t>
+  </si>
+  <si>
     <t>Referral name</t>
   </si>
   <si>
-    <t>ABC HOSPITAL</t>
+    <t>AEH - ANDIPATTI</t>
   </si>
   <si>
     <t>Clinic Referred to</t>
@@ -235,44 +259,109 @@
     <t xml:space="preserve">UNIT-1 </t>
   </si>
   <si>
+    <t xml:space="preserve">UNIT-2 </t>
+  </si>
+  <si>
     <t>Doctor Referred to</t>
   </si>
   <si>
     <t>Anu N V</t>
+  </si>
+  <si>
+    <t>Referral name from vision center</t>
+  </si>
+  <si>
+    <t>AEH - THIRUCHULI</t>
+  </si>
+  <si>
+    <t>Referral name from community center</t>
+  </si>
+  <si>
+    <t>AEH - THIRUMANGALAM</t>
+  </si>
+  <si>
+    <t>ConcessionApprovedBy</t>
+  </si>
+  <si>
+    <t>Concession granted</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>Concession Reason</t>
+  </si>
+  <si>
+    <t>Concession remarks</t>
+  </si>
+  <si>
+    <t>Concession remarks are entered</t>
+  </si>
+  <si>
+    <t>Clinic Referred to Free or Camp</t>
+  </si>
+  <si>
+    <t>FREENEW</t>
+  </si>
+  <si>
+    <t>PaymentType</t>
+  </si>
+  <si>
+    <t>CASH</t>
+  </si>
+  <si>
+    <t>HOSPITAL ACCOUNT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Bad" xfId="1" builtinId="27"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0"/>
@@ -572,318 +661,524 @@
   <cols>
     <col min="1" max="1" width="39.28516" customWidth="1"/>
     <col min="2" max="2" width="40.28516" customWidth="1"/>
+    <col min="3" max="3" width="31.28516" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="1">
+        <v>9</v>
+      </c>
+      <c r="B5" s="2">
+        <v>25</v>
+      </c>
+      <c r="C5" s="2">
         <v>25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" s="1">
+        <v>32</v>
+      </c>
+      <c r="B16" s="2">
+        <v>645126</v>
+      </c>
+      <c r="C16" s="2">
         <v>645126</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>32</v>
-      </c>
-      <c r="B18" s="1">
+        <v>35</v>
+      </c>
+      <c r="B18" s="2">
+        <v>8457962513</v>
+      </c>
+      <c r="C18" s="2">
         <v>8457962513</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>33</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>35</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>37</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>39</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="s">
-        <v>41</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>42</v>
+      <c r="A23" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>43</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>45</v>
-      </c>
-      <c r="B25" s="1">
+        <v>48</v>
+      </c>
+      <c r="B25" s="2">
+        <v>50</v>
+      </c>
+      <c r="C25" s="2">
         <v>50</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>46</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>48</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="s">
-        <v>50</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>51</v>
+      <c r="A28" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>52</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>54</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>56</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>58</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>60</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>62</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>63</v>
+        <v>68</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>64</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>66</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>67</v>
+        <v>73</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>68</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>69</v>
+        <v>76</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>70</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>71</v>
+        <v>78</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>72</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>73</v>
+        <v>81</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>83</v>
+      </c>
+      <c r="B40" t="s">
+        <v>84</v>
+      </c>
+      <c r="C40" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>85</v>
+      </c>
+      <c r="B41" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>87</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>88</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>91</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>92</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>94</v>
+      </c>
+      <c r="B46" t="s">
+        <v>95</v>
+      </c>
+      <c r="C46" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B47" t="s">
+        <v>97</v>
+      </c>
+      <c r="C47" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completed Multiple patient data integration
</commit_message>
<xml_diff>
--- a/demoplay/src/test/resources/OPRegistrationDataJsonValidation.xlsx
+++ b/demoplay/src/test/resources/OPRegistrationDataJsonValidation.xlsx
@@ -28,6 +28,9 @@
     <t>FREE</t>
   </si>
   <si>
+    <t>CAMP</t>
+  </si>
+  <si>
     <t>PatientType</t>
   </si>
   <si>
@@ -37,7 +40,13 @@
     <t>FirstName</t>
   </si>
   <si>
-    <t>AAA</t>
+    <t>PPPP</t>
+  </si>
+  <si>
+    <t>FFFF</t>
+  </si>
+  <si>
+    <t>CCCC</t>
   </si>
   <si>
     <t>LastName</t>
@@ -49,6 +58,9 @@
     <t>Age</t>
   </si>
   <si>
+    <t>24</t>
+  </si>
+  <si>
     <t>Date of Birth</t>
   </si>
   <si>
@@ -64,24 +76,102 @@
     <t>Female</t>
   </si>
   <si>
+    <t>Male</t>
+  </si>
+  <si>
     <t>NextOfKinType</t>
   </si>
   <si>
     <t>D/O</t>
   </si>
   <si>
+    <t>S/O</t>
+  </si>
+  <si>
     <t>NextOfKinName</t>
   </si>
   <si>
     <t>sss</t>
   </si>
   <si>
+    <t>iii</t>
+  </si>
+  <si>
     <t>ReferralType</t>
   </si>
   <si>
+    <t>Referral</t>
+  </si>
+  <si>
     <t>Normal</t>
   </si>
   <si>
+    <t>Reference No</t>
+  </si>
+  <si>
+    <t>12563</t>
+  </si>
+  <si>
+    <t>12564</t>
+  </si>
+  <si>
+    <t>12565</t>
+  </si>
+  <si>
+    <t>Reference date</t>
+  </si>
+  <si>
+    <t>20-06-2026</t>
+  </si>
+  <si>
+    <t>20-06-2027</t>
+  </si>
+  <si>
+    <t>20-06-2028</t>
+  </si>
+  <si>
+    <t>Referral name</t>
+  </si>
+  <si>
+    <t>AEH - ANDIPATTI</t>
+  </si>
+  <si>
+    <t>Clinic Referred to</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIT-1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIT-2 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIT-3 </t>
+  </si>
+  <si>
+    <t>Doctor Referred to</t>
+  </si>
+  <si>
+    <t>Anu N V</t>
+  </si>
+  <si>
+    <t>Referral name from vision center</t>
+  </si>
+  <si>
+    <t>AEH - THIRUCHULI</t>
+  </si>
+  <si>
+    <t>Referral name from community center</t>
+  </si>
+  <si>
+    <t>AEH - THIRUMANGALAM</t>
+  </si>
+  <si>
+    <t>Clinic Referred to Free or Camp</t>
+  </si>
+  <si>
+    <t>FREENEW</t>
+  </si>
+  <si>
     <t>Nationality</t>
   </si>
   <si>
@@ -97,6 +187,9 @@
     <t>99 rrr street</t>
   </si>
   <si>
+    <t>100 rrr street</t>
+  </si>
+  <si>
     <t>locality</t>
   </si>
   <si>
@@ -157,6 +250,9 @@
     <t>Concession</t>
   </si>
   <si>
+    <t>Subsidy</t>
+  </si>
+  <si>
     <t>SubsidyApprovedBy</t>
   </si>
   <si>
@@ -178,12 +274,39 @@
     <t>Subsidy remarks are entered</t>
   </si>
   <si>
+    <t>ConcessionApprovedBy</t>
+  </si>
+  <si>
+    <t>Concession granted</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>Concession Reason</t>
+  </si>
+  <si>
+    <t>Concession remarks</t>
+  </si>
+  <si>
+    <t>Concession remarks are entered</t>
+  </si>
+  <si>
     <t>Patient category</t>
   </si>
   <si>
     <t>FULL PAYMENT</t>
   </si>
   <si>
+    <t>CORPORATE</t>
+  </si>
+  <si>
     <t>Corporate name</t>
   </si>
   <si>
@@ -199,6 +322,9 @@
     <t>458968</t>
   </si>
   <si>
+    <t>458969</t>
+  </si>
+  <si>
     <t>Employee grade</t>
   </si>
   <si>
@@ -214,6 +340,9 @@
     <t>1523445</t>
   </si>
   <si>
+    <t>4573239</t>
+  </si>
+  <si>
     <t>Claim id</t>
   </si>
   <si>
@@ -223,88 +352,13 @@
     <t>3048342</t>
   </si>
   <si>
+    <t>6098136</t>
+  </si>
+  <si>
     <t>Corporate remarks</t>
   </si>
   <si>
     <t>Corporate remarks is entered</t>
-  </si>
-  <si>
-    <t>Reference No</t>
-  </si>
-  <si>
-    <t>12563</t>
-  </si>
-  <si>
-    <t>12564</t>
-  </si>
-  <si>
-    <t>Reference date</t>
-  </si>
-  <si>
-    <t>20-06-2026</t>
-  </si>
-  <si>
-    <t>20-06-2027</t>
-  </si>
-  <si>
-    <t>Referral name</t>
-  </si>
-  <si>
-    <t>AEH - ANDIPATTI</t>
-  </si>
-  <si>
-    <t>Clinic Referred to</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIT-1 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIT-2 </t>
-  </si>
-  <si>
-    <t>Doctor Referred to</t>
-  </si>
-  <si>
-    <t>Anu N V</t>
-  </si>
-  <si>
-    <t>Referral name from vision center</t>
-  </si>
-  <si>
-    <t>AEH - THIRUCHULI</t>
-  </si>
-  <si>
-    <t>Referral name from community center</t>
-  </si>
-  <si>
-    <t>AEH - THIRUMANGALAM</t>
-  </si>
-  <si>
-    <t>ConcessionApprovedBy</t>
-  </si>
-  <si>
-    <t>Concession granted</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>Concession Reason</t>
-  </si>
-  <si>
-    <t>Concession remarks</t>
-  </si>
-  <si>
-    <t>Concession remarks are entered</t>
-  </si>
-  <si>
-    <t>Clinic Referred to Free or Camp</t>
-  </si>
-  <si>
-    <t>FREENEW</t>
   </si>
   <si>
     <t>PaymentType</t>
@@ -354,10 +408,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -662,6 +717,7 @@
     <col min="1" max="1" width="39.28516" customWidth="1"/>
     <col min="2" max="2" width="40.28516" customWidth="1"/>
     <col min="3" max="3" width="31.28516" customWidth="1"/>
+    <col min="4" max="4" width="28.71094" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -674,43 +730,55 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2">
         <v>25</v>
@@ -718,468 +786,607 @@
       <c r="C5" s="2">
         <v>25</v>
       </c>
+      <c r="D5" s="2" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>18</v>
+        <v>24</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="s">
-        <v>19</v>
+      <c r="A10" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>20</v>
+        <v>28</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>22</v>
+        <v>31</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>25</v>
+        <v>35</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>27</v>
+        <v>38</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>29</v>
+        <v>41</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>31</v>
+        <v>44</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="2">
-        <v>645126</v>
-      </c>
-      <c r="C16" s="2">
-        <v>645126</v>
+        <v>45</v>
+      </c>
+      <c r="B16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>33</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>34</v>
+        <v>47</v>
+      </c>
+      <c r="B17" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>35</v>
-      </c>
-      <c r="B18" s="2">
-        <v>8457962513</v>
-      </c>
-      <c r="C18" s="2">
-        <v>8457962513</v>
+        <v>49</v>
+      </c>
+      <c r="B18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>37</v>
+        <v>52</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>39</v>
+        <v>55</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>41</v>
+        <v>58</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>43</v>
+        <v>60</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="s">
-        <v>44</v>
+      <c r="A23" t="s">
+        <v>61</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>45</v>
+        <v>62</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>46</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>47</v>
+        <v>63</v>
+      </c>
+      <c r="B24" s="2">
+        <v>645126</v>
+      </c>
+      <c r="C24" s="2">
+        <v>645126</v>
+      </c>
+      <c r="D24" s="2">
+        <v>645126</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>48</v>
-      </c>
-      <c r="B25" s="2">
-        <v>50</v>
-      </c>
-      <c r="C25" s="2">
-        <v>50</v>
+        <v>64</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>49</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>50</v>
+        <v>66</v>
+      </c>
+      <c r="B26" s="2">
+        <v>8457962513</v>
+      </c>
+      <c r="C26" s="2">
+        <v>8457962513</v>
+      </c>
+      <c r="D26" s="2">
+        <v>8457962513</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>52</v>
+        <v>68</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="s">
-        <v>53</v>
+      <c r="A28" t="s">
+        <v>69</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>2</v>
+        <v>70</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>56</v>
+        <v>72</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>59</v>
+        <v>74</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="s">
-        <v>60</v>
+      <c r="A31" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>61</v>
+        <v>77</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>64</v>
+        <v>79</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>65</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>67</v>
+        <v>80</v>
+      </c>
+      <c r="B33" s="2">
+        <v>50</v>
+      </c>
+      <c r="C33" s="2">
+        <v>50</v>
+      </c>
+      <c r="D33" s="2">
+        <v>50</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>69</v>
+        <v>82</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>72</v>
+        <v>84</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>77</v>
+        <v>88</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>82</v>
+        <v>92</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="s">
-        <v>83</v>
-      </c>
-      <c r="B40" t="s">
-        <v>84</v>
-      </c>
-      <c r="C40" t="s">
-        <v>84</v>
+      <c r="A40" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>85</v>
-      </c>
-      <c r="B41" t="s">
-        <v>86</v>
-      </c>
-      <c r="C41" t="s">
-        <v>86</v>
+        <v>96</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>47</v>
+        <v>99</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>47</v>
+        <v>100</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>90</v>
+        <v>103</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>50</v>
+        <v>105</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>50</v>
+        <v>106</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>93</v>
+        <v>110</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>94</v>
-      </c>
-      <c r="B46" t="s">
-        <v>95</v>
-      </c>
-      <c r="C46" t="s">
-        <v>95</v>
+        <v>112</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="B47" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C47" t="s">
-        <v>98</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="D47" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+    </row>
+    <row r="57">
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
Payment type Other Initial commit
</commit_message>
<xml_diff>
--- a/demoplay/src/test/resources/OPRegistrationDataJsonValidation.xlsx
+++ b/demoplay/src/test/resources/OPRegistrationDataJsonValidation.xlsx
@@ -100,12 +100,12 @@
     <t>ReferralType</t>
   </si>
   <si>
+    <t>Normal</t>
+  </si>
+  <si>
     <t>Referral</t>
   </si>
   <si>
-    <t>Normal</t>
-  </si>
-  <si>
     <t>Reference No</t>
   </si>
   <si>
@@ -247,12 +247,12 @@
     <t>PatientSubCategory</t>
   </si>
   <si>
+    <t>Subsidy</t>
+  </si>
+  <si>
     <t>Concession</t>
   </si>
   <si>
-    <t>Subsidy</t>
-  </si>
-  <si>
     <t>SubsidyApprovedBy</t>
   </si>
   <si>
@@ -280,15 +280,15 @@
     <t>Concession granted</t>
   </si>
   <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
     <t>30</t>
   </si>
   <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
     <t>Concession Reason</t>
   </si>
   <si>
@@ -307,6 +307,9 @@
     <t>CORPORATE</t>
   </si>
   <si>
+    <t>VISION CENTER</t>
+  </si>
+  <si>
     <t>Corporate name</t>
   </si>
   <si>
@@ -364,10 +367,22 @@
     <t>PaymentType</t>
   </si>
   <si>
+    <t>OTHERS</t>
+  </si>
+  <si>
+    <t>HOSPITAL ACCOUNT</t>
+  </si>
+  <si>
     <t>CASH</t>
   </si>
   <si>
-    <t>HOSPITAL ACCOUNT</t>
+    <t>selectCounter</t>
+  </si>
+  <si>
+    <t>Orbit</t>
+  </si>
+  <si>
+    <t>Cornea</t>
   </si>
 </sst>
 </file>
@@ -408,11 +423,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -718,6 +732,7 @@
     <col min="2" max="2" width="40.28516" customWidth="1"/>
     <col min="3" max="3" width="31.28516" customWidth="1"/>
     <col min="4" max="4" width="28.71094" customWidth="1"/>
+    <col min="5" max="5" width="28.71094" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -733,6 +748,9 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -747,6 +765,9 @@
       <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -761,6 +782,9 @@
       <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="E3" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
@@ -775,6 +799,9 @@
       <c r="D4" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="E4" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
@@ -789,6 +816,9 @@
       <c r="D5" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="E5" s="2">
+        <v>25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
@@ -803,6 +833,9 @@
       <c r="D6" s="2" t="s">
         <v>16</v>
       </c>
+      <c r="E6" s="2" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
@@ -817,6 +850,9 @@
       <c r="D7" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="E7" s="2" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
@@ -831,6 +867,9 @@
       <c r="D8" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="E8" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
@@ -845,9 +884,12 @@
       <c r="D9" s="2" t="s">
         <v>25</v>
       </c>
+      <c r="E9" s="2" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -857,7 +899,10 @@
         <v>28</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="11">
@@ -873,6 +918,9 @@
       <c r="D11" s="2" t="s">
         <v>32</v>
       </c>
+      <c r="E11" s="2" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
@@ -887,6 +935,9 @@
       <c r="D12" s="2" t="s">
         <v>36</v>
       </c>
+      <c r="E12" s="2" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
@@ -901,6 +952,9 @@
       <c r="D13" s="2" t="s">
         <v>38</v>
       </c>
+      <c r="E13" s="2" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
@@ -915,6 +969,9 @@
       <c r="D14" s="2" t="s">
         <v>42</v>
       </c>
+      <c r="E14" s="2" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
@@ -929,6 +986,9 @@
       <c r="D15" s="2" t="s">
         <v>44</v>
       </c>
+      <c r="E15" s="2" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
@@ -943,6 +1003,9 @@
       <c r="D16" t="s">
         <v>46</v>
       </c>
+      <c r="E16" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
@@ -957,6 +1020,9 @@
       <c r="D17" t="s">
         <v>48</v>
       </c>
+      <c r="E17" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
@@ -971,6 +1037,9 @@
       <c r="D18" t="s">
         <v>50</v>
       </c>
+      <c r="E18" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
@@ -985,6 +1054,9 @@
       <c r="D19" s="2" t="s">
         <v>52</v>
       </c>
+      <c r="E19" s="2" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
@@ -999,6 +1071,9 @@
       <c r="D20" s="2" t="s">
         <v>56</v>
       </c>
+      <c r="E20" s="2" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
@@ -1013,6 +1088,9 @@
       <c r="D21" s="2" t="s">
         <v>58</v>
       </c>
+      <c r="E21" s="2" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
@@ -1027,6 +1105,9 @@
       <c r="D22" s="2" t="s">
         <v>60</v>
       </c>
+      <c r="E22" s="2" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
@@ -1041,6 +1122,9 @@
       <c r="D23" s="2" t="s">
         <v>62</v>
       </c>
+      <c r="E23" s="2" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
@@ -1055,6 +1139,9 @@
       <c r="D24" s="2">
         <v>645126</v>
       </c>
+      <c r="E24" s="2">
+        <v>645126</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
@@ -1069,6 +1156,9 @@
       <c r="D25" s="2" t="s">
         <v>65</v>
       </c>
+      <c r="E25" s="2" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
@@ -1083,6 +1173,9 @@
       <c r="D26" s="2">
         <v>8457962513</v>
       </c>
+      <c r="E26" s="2">
+        <v>8457962513</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
@@ -1097,6 +1190,9 @@
       <c r="D27" s="2" t="s">
         <v>68</v>
       </c>
+      <c r="E27" s="2" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
@@ -1111,6 +1207,9 @@
       <c r="D28" s="2" t="s">
         <v>70</v>
       </c>
+      <c r="E28" s="2" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
@@ -1125,6 +1224,9 @@
       <c r="D29" s="2" t="s">
         <v>72</v>
       </c>
+      <c r="E29" s="2" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
@@ -1139,18 +1241,22 @@
       <c r="D30" s="2" t="s">
         <v>74</v>
       </c>
+      <c r="E30" s="2" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="2"/>
+      <c r="C31" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="D31" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1158,13 +1264,14 @@
       <c r="A32" t="s">
         <v>78</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>79</v>
-      </c>
+      <c r="B32" s="2"/>
       <c r="C32" s="2" t="s">
         <v>79</v>
       </c>
       <c r="D32" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1172,13 +1279,14 @@
       <c r="A33" t="s">
         <v>80</v>
       </c>
-      <c r="B33" s="2">
-        <v>50</v>
-      </c>
+      <c r="B33" s="2"/>
       <c r="C33" s="2">
         <v>50</v>
       </c>
       <c r="D33" s="2">
+        <v>50</v>
+      </c>
+      <c r="E33" s="2">
         <v>50</v>
       </c>
     </row>
@@ -1186,13 +1294,14 @@
       <c r="A34" t="s">
         <v>81</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>82</v>
-      </c>
+      <c r="B34" s="2"/>
       <c r="C34" s="2" t="s">
         <v>82</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>82</v>
       </c>
     </row>
@@ -1200,13 +1309,14 @@
       <c r="A35" t="s">
         <v>83</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>84</v>
-      </c>
+      <c r="B35" s="2"/>
       <c r="C35" s="2" t="s">
         <v>84</v>
       </c>
       <c r="D35" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1214,13 +1324,14 @@
       <c r="A36" t="s">
         <v>85</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>79</v>
-      </c>
+      <c r="B36" s="2"/>
       <c r="C36" s="2" t="s">
         <v>79</v>
       </c>
       <c r="D36" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1228,13 +1339,14 @@
       <c r="A37" t="s">
         <v>86</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="2"/>
+      <c r="C37" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="D37" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="E37" s="2" t="s">
         <v>89</v>
       </c>
     </row>
@@ -1242,13 +1354,14 @@
       <c r="A38" t="s">
         <v>90</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>82</v>
-      </c>
+      <c r="B38" s="2"/>
       <c r="C38" s="2" t="s">
         <v>82</v>
       </c>
       <c r="D38" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E38" s="2" t="s">
         <v>82</v>
       </c>
     </row>
@@ -1256,13 +1369,14 @@
       <c r="A39" t="s">
         <v>91</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>92</v>
-      </c>
+      <c r="B39" s="2"/>
       <c r="C39" s="2" t="s">
         <v>92</v>
       </c>
       <c r="D39" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E39" s="2" t="s">
         <v>92</v>
       </c>
     </row>
@@ -1279,103 +1393,138 @@
       <c r="D40" s="2" t="s">
         <v>95</v>
       </c>
+      <c r="E40" s="2" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E42" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E44" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B47" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C47" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D47" t="s">
-        <v>116</v>
+        <v>117</v>
+      </c>
+      <c r="E47" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>119</v>
+      </c>
+      <c r="B48" t="s">
+        <v>120</v>
+      </c>
+      <c r="E48" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="56">

</xml_diff>

<commit_message>
View collection, Reprint, Recall, Unit Load, Route card
</commit_message>
<xml_diff>
--- a/demoplay/src/test/resources/OPRegistrationDataJsonValidation.xlsx
+++ b/demoplay/src/test/resources/OPRegistrationDataJsonValidation.xlsx
@@ -7,18 +7,19 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="opRegistrationData" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="datas" sheetId="2" r:id="rId2"/>
+    <sheet name="Extra collection" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="2">
   <si>
     <t>PayFree</t>
   </si>
@@ -200,231 +201,240 @@
     <t>PatientSubCategory</t>
   </si>
   <si>
+    <t>SubsidyApprovedBy</t>
+  </si>
+  <si>
+    <t>AEH-DINDIGUL</t>
+  </si>
+  <si>
+    <t>Subsidy granted</t>
+  </si>
+  <si>
+    <t>Subsidy Reason</t>
+  </si>
+  <si>
+    <t>CAMP SUBSIDY</t>
+  </si>
+  <si>
+    <t>Subsidy remarks</t>
+  </si>
+  <si>
+    <t>Subsidy remarks are entered</t>
+  </si>
+  <si>
+    <t>ConcessionApprovedBy</t>
+  </si>
+  <si>
+    <t>Concession granted</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>Concession Reason</t>
+  </si>
+  <si>
+    <t>Concession remarks</t>
+  </si>
+  <si>
+    <t>Concession remarks are entered</t>
+  </si>
+  <si>
+    <t>Patient category</t>
+  </si>
+  <si>
+    <t>FULL PAYMENT</t>
+  </si>
+  <si>
+    <t>Corporate name</t>
+  </si>
+  <si>
+    <t>NIND STUDY</t>
+  </si>
+  <si>
+    <t>Document Ref.no</t>
+  </si>
+  <si>
+    <t>458967</t>
+  </si>
+  <si>
+    <t>Employee grade</t>
+  </si>
+  <si>
+    <t>EMPLOYEE</t>
+  </si>
+  <si>
+    <t>Employee code</t>
+  </si>
+  <si>
+    <t>1526349</t>
+  </si>
+  <si>
+    <t>Claim id</t>
+  </si>
+  <si>
+    <t>1452</t>
+  </si>
+  <si>
+    <t>Corporate remarks</t>
+  </si>
+  <si>
+    <t>Corporate remarks is entered</t>
+  </si>
+  <si>
+    <t>PaymentType</t>
+  </si>
+  <si>
+    <t>CASH</t>
+  </si>
+  <si>
+    <t>selectCounter</t>
+  </si>
+  <si>
+    <t>Cornea</t>
+  </si>
+  <si>
+    <t>Foreign country</t>
+  </si>
+  <si>
+    <t>AFRICA</t>
+  </si>
+  <si>
+    <t>zip code</t>
+  </si>
+  <si>
+    <t>5464</t>
+  </si>
+  <si>
+    <t>REPRINT</t>
+  </si>
+  <si>
+    <t>PatientTypeReprint</t>
+  </si>
+  <si>
+    <t>dateReprint</t>
+  </si>
+  <si>
+    <t>22-07-2026</t>
+  </si>
+  <si>
+    <t>uinReprint</t>
+  </si>
+  <si>
+    <t>0024427414</t>
+  </si>
+  <si>
+    <t>ReprintChoice</t>
+  </si>
+  <si>
+    <t>ID Card</t>
+  </si>
+  <si>
+    <t>ReceiptReprint</t>
+  </si>
+  <si>
+    <t>uinRouteCard</t>
+  </si>
+  <si>
+    <t>MRN</t>
+  </si>
+  <si>
+    <t>P6089-554</t>
+  </si>
+  <si>
+    <t>UIN</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>UNIT-3</t>
+  </si>
+  <si>
+    <t>FREE</t>
+  </si>
+  <si>
+    <t>CAMP</t>
+  </si>
+  <si>
+    <t>FFFF</t>
+  </si>
+  <si>
+    <t>CCCC</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>25-06-2001</t>
+  </si>
+  <si>
+    <t>25-06-2002</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>S/O</t>
+  </si>
+  <si>
+    <t>iii</t>
+  </si>
+  <si>
+    <t>Referral</t>
+  </si>
+  <si>
+    <t>12564</t>
+  </si>
+  <si>
+    <t>12565</t>
+  </si>
+  <si>
+    <t>20-06-2027</t>
+  </si>
+  <si>
+    <t>20-06-2028</t>
+  </si>
+  <si>
+    <t>07-07-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIT-2 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIT-3 </t>
+  </si>
+  <si>
+    <t>Indian</t>
+  </si>
+  <si>
+    <t>99 rrr street</t>
+  </si>
+  <si>
+    <t>100 rrr street</t>
+  </si>
+  <si>
+    <t>7851200369</t>
+  </si>
+  <si>
+    <t>emailihms02@gmail.com</t>
+  </si>
+  <si>
+    <t>Subsidy</t>
+  </si>
+  <si>
     <t>Concession</t>
   </si>
   <si>
-    <t>SubsidyApprovedBy</t>
-  </si>
-  <si>
-    <t>AEH-DINDIGUL</t>
-  </si>
-  <si>
-    <t>Subsidy granted</t>
-  </si>
-  <si>
-    <t>Subsidy Reason</t>
-  </si>
-  <si>
-    <t>CAMP SUBSIDY</t>
-  </si>
-  <si>
-    <t>Subsidy remarks</t>
-  </si>
-  <si>
-    <t>Subsidy remarks are entered</t>
-  </si>
-  <si>
-    <t>ConcessionApprovedBy</t>
-  </si>
-  <si>
-    <t>Concession granted</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>Concession Reason</t>
-  </si>
-  <si>
-    <t>Concession remarks</t>
-  </si>
-  <si>
-    <t>Concession remarks are entered</t>
-  </si>
-  <si>
-    <t>Patient category</t>
+    <t>31</t>
+  </si>
+  <si>
+    <t>32</t>
   </si>
   <si>
     <t>CORPORATE</t>
   </si>
   <si>
-    <t>Corporate name</t>
-  </si>
-  <si>
-    <t>NIND STUDY</t>
-  </si>
-  <si>
-    <t>Document Ref.no</t>
-  </si>
-  <si>
-    <t>458967</t>
-  </si>
-  <si>
-    <t>Employee grade</t>
-  </si>
-  <si>
-    <t>EMPLOYEE</t>
-  </si>
-  <si>
-    <t>Employee code</t>
-  </si>
-  <si>
-    <t>1526349</t>
-  </si>
-  <si>
-    <t>Claim id</t>
-  </si>
-  <si>
-    <t>1452</t>
-  </si>
-  <si>
-    <t>Corporate remarks</t>
-  </si>
-  <si>
-    <t>Corporate remarks is entered</t>
-  </si>
-  <si>
-    <t>PaymentType</t>
-  </si>
-  <si>
-    <t>CASH</t>
-  </si>
-  <si>
-    <t>selectCounter</t>
-  </si>
-  <si>
-    <t>Cornea</t>
-  </si>
-  <si>
-    <t>Foreign country</t>
-  </si>
-  <si>
-    <t>AFRICA</t>
-  </si>
-  <si>
-    <t>zip code</t>
-  </si>
-  <si>
-    <t>5464</t>
-  </si>
-  <si>
-    <t>REPRINT</t>
-  </si>
-  <si>
-    <t>PatientTypeReprint</t>
-  </si>
-  <si>
-    <t>dateReprint</t>
-  </si>
-  <si>
-    <t>uinReprint</t>
-  </si>
-  <si>
-    <t>ReprintChoice</t>
-  </si>
-  <si>
-    <t>ReceiptReprint</t>
-  </si>
-  <si>
-    <t>MRN</t>
-  </si>
-  <si>
-    <t>P6089-522</t>
-  </si>
-  <si>
-    <t>UIN</t>
-  </si>
-  <si>
-    <t>0024427367</t>
-  </si>
-  <si>
-    <t>Location</t>
-  </si>
-  <si>
-    <t>UNIT-3</t>
-  </si>
-  <si>
-    <t>FREE</t>
-  </si>
-  <si>
-    <t>CAMP</t>
-  </si>
-  <si>
-    <t>FFFF</t>
-  </si>
-  <si>
-    <t>CCCC</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>25-06-2001</t>
-  </si>
-  <si>
-    <t>25-06-2002</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>S/O</t>
-  </si>
-  <si>
-    <t>iii</t>
-  </si>
-  <si>
-    <t>Referral</t>
-  </si>
-  <si>
-    <t>12564</t>
-  </si>
-  <si>
-    <t>12565</t>
-  </si>
-  <si>
-    <t>20-06-2027</t>
-  </si>
-  <si>
-    <t>20-06-2028</t>
-  </si>
-  <si>
-    <t>07-07-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIT-2 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIT-3 </t>
-  </si>
-  <si>
-    <t>Indian</t>
-  </si>
-  <si>
-    <t>99 rrr street</t>
-  </si>
-  <si>
-    <t>100 rrr street</t>
-  </si>
-  <si>
-    <t>7851200369</t>
-  </si>
-  <si>
-    <t>emailihms02@gmail.com</t>
-  </si>
-  <si>
-    <t>Subsidy</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>FULL PAYMENT</t>
-  </si>
-  <si>
     <t>458968</t>
   </si>
   <si>
@@ -455,9 +465,6 @@
     <t>0024427261</t>
   </si>
   <si>
-    <t>ID Card</t>
-  </si>
-  <si>
     <t>O26271735 - 20/07/2026</t>
   </si>
   <si>
@@ -473,10 +480,20 @@
     <t>0024427271</t>
   </si>
   <si>
-    <t>P6089-526</t>
-  </si>
-  <si>
-    <t>0024427371</t>
+    <t>Total Collection Registration</t>
+  </si>
+  <si>
+    <t>₹ 1600</t>
+  </si>
+  <si>
+    <t>Unit Load Registration</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>New Patients Allotted To | UNIT-1 = 10  | UNIT-2 = 9  | UNIT-3 = 29 
+Actual Overall Patients | UNIT-1 = 10  | UNIT-2 = 12  | UNIT-3 = 28</t>
   </si>
 </sst>
 </file>
@@ -835,7 +852,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="39.28516"/>
@@ -1089,21 +1106,19 @@
       <c r="A31" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>60</v>
-      </c>
+      <c r="B31" s="2"/>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B33" s="2">
         <v>50</v>
@@ -1111,152 +1126,158 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B47" t="s" s="0">
         <v>88</v>
-      </c>
-      <c r="B47" t="s" s="0">
-        <v>89</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="B48" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="B48" t="s" s="0">
-        <v>91</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="B49" t="s" s="0">
         <v>92</v>
-      </c>
-      <c r="B49" t="s" s="0">
-        <v>93</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
+        <v>93</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>97</v>
+        <v>96</v>
+      </c>
+      <c r="B52" t="s" s="0">
+        <v>54</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
+        <v>97</v>
+      </c>
+      <c r="B53" t="s" s="0">
         <v>98</v>
       </c>
     </row>
@@ -1264,45 +1285,59 @@
       <c r="A54" t="s" s="0">
         <v>99</v>
       </c>
+      <c r="B54" s="2" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>100</v>
+        <v>101</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>102</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>102</v>
-      </c>
-      <c r="B57" t="s" s="0">
-        <v>151</v>
+        <v>104</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>152</v>
+        <v>106</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D59" s="2"/>
+        <v>100</v>
+      </c>
     </row>
     <row r="60">
-      <c r="C60" s="2"/>
+      <c r="A60" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>109</v>
+      </c>
       <c r="D60" s="2"/>
+    </row>
+    <row r="61">
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
     </row>
   </sheetData>
 </worksheet>
@@ -1321,10 +1356,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -1349,10 +1384,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>5</v>
@@ -1378,7 +1413,7 @@
         <v>25</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C5" s="2">
         <v>25</v>
@@ -1389,13 +1424,13 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>11</v>
@@ -1406,13 +1441,13 @@
         <v>13</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8">
@@ -1420,13 +1455,13 @@
         <v>15</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9">
@@ -1434,7 +1469,7 @@
         <v>17</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>17</v>
@@ -1445,7 +1480,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>19</v>
@@ -1459,10 +1494,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>21</v>
@@ -1473,16 +1508,16 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13">
@@ -1501,10 +1536,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>27</v>
@@ -1571,24 +1606,24 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>39</v>
@@ -1659,7 +1694,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B26" s="2">
         <v>8457962513</v>
@@ -1673,7 +1708,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>52</v>
@@ -1727,25 +1762,25 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>60</v>
+        <v>134</v>
       </c>
       <c r="D31" s="2"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D32" s="2"/>
     </row>
@@ -1763,194 +1798,194 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D34" s="2"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D35" s="2"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D36" s="2"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D37" s="2"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D38" s="2"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D39" s="2"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>75</v>
+        <v>137</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>75</v>
+        <v>137</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>134</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C47" t="s" s="0">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="48">
       <c r="C48" t="s" s="0">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="50">
@@ -1960,38 +1995,38 @@
     </row>
     <row r="51">
       <c r="D51" t="s" s="0">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="52">
       <c r="D52" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="53">
       <c r="D53" t="s" s="0">
-        <v>145</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54">
       <c r="D54" t="s" s="0">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="57">
@@ -1999,7 +2034,35 @@
         <v>35</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="33.0"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>153</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>155</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Biling until Test enter, Edit address, patient information, patient enquiry (initial)
</commit_message>
<xml_diff>
--- a/demoplay/src/test/resources/OPRegistrationDataJsonValidation.xlsx
+++ b/demoplay/src/test/resources/OPRegistrationDataJsonValidation.xlsx
@@ -7,7 +7,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="opRegistrationData" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>PayFree</t>
   </si>
@@ -52,6 +52,9 @@
     <t>26</t>
   </si>
   <si>
+    <t>27</t>
+  </si>
+  <si>
     <t>Date of Birth</t>
   </si>
   <si>
@@ -91,12 +94,18 @@
     <t>12563</t>
   </si>
   <si>
+    <t>12564</t>
+  </si>
+  <si>
     <t>Reference date</t>
   </si>
   <si>
     <t>20-06-2026</t>
   </si>
   <si>
+    <t>20-06-2027</t>
+  </si>
+  <si>
     <t>Referral name</t>
   </si>
   <si>
@@ -109,6 +118,9 @@
     <t xml:space="preserve">UNIT-1 </t>
   </si>
   <si>
+    <t xml:space="preserve">UNIT-2 </t>
+  </si>
+  <si>
     <t>Doctor Referred to</t>
   </si>
   <si>
@@ -139,331 +151,319 @@
     <t>Foreigner</t>
   </si>
   <si>
+    <t>DoorStreet</t>
+  </si>
+  <si>
+    <t>98 rrr street</t>
+  </si>
+  <si>
+    <t>99 rrr street</t>
+  </si>
+  <si>
+    <t>locality</t>
+  </si>
+  <si>
+    <t>inside madurai</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>madurai</t>
+  </si>
+  <si>
+    <t>Area</t>
+  </si>
+  <si>
+    <t>BEE BEE KULAM</t>
+  </si>
+  <si>
+    <t>PinCode</t>
+  </si>
+  <si>
+    <t>Taluk</t>
+  </si>
+  <si>
+    <t>MADURAI - GENL</t>
+  </si>
+  <si>
+    <t>MobileNo</t>
+  </si>
+  <si>
+    <t>6854120032</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>emailihms49@gmail.com</t>
+  </si>
+  <si>
+    <t>PurposeVisit</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>ConsentForm</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Assign doctor</t>
+  </si>
+  <si>
+    <t>Esha</t>
+  </si>
+  <si>
+    <t>PatientSubCategory</t>
+  </si>
+  <si>
+    <t>SubsidyApprovedBy</t>
+  </si>
+  <si>
+    <t>AEH-DINDIGUL</t>
+  </si>
+  <si>
+    <t>Subsidy granted</t>
+  </si>
+  <si>
+    <t>Subsidy Reason</t>
+  </si>
+  <si>
+    <t>CAMP SUBSIDY</t>
+  </si>
+  <si>
+    <t>Subsidy remarks</t>
+  </si>
+  <si>
+    <t>Subsidy remarks are entered</t>
+  </si>
+  <si>
+    <t>ConcessionApprovedBy</t>
+  </si>
+  <si>
+    <t>Concession granted</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>Concession Reason</t>
+  </si>
+  <si>
+    <t>Concession remarks</t>
+  </si>
+  <si>
+    <t>Concession remarks are entered</t>
+  </si>
+  <si>
+    <t>Patient category</t>
+  </si>
+  <si>
+    <t>FULL PAYMENT</t>
+  </si>
+  <si>
+    <t>Corporate name</t>
+  </si>
+  <si>
+    <t>NIND STUDY</t>
+  </si>
+  <si>
+    <t>Document Ref.no</t>
+  </si>
+  <si>
+    <t>458967</t>
+  </si>
+  <si>
+    <t>458968</t>
+  </si>
+  <si>
+    <t>Employee grade</t>
+  </si>
+  <si>
+    <t>EMPLOYEE</t>
+  </si>
+  <si>
+    <t>Employee code</t>
+  </si>
+  <si>
+    <t>1526349</t>
+  </si>
+  <si>
+    <t>1523445</t>
+  </si>
+  <si>
+    <t>Claim id</t>
+  </si>
+  <si>
+    <t>1452</t>
+  </si>
+  <si>
+    <t>3048342</t>
+  </si>
+  <si>
+    <t>Corporate remarks</t>
+  </si>
+  <si>
+    <t>Corporate remarks is entered</t>
+  </si>
+  <si>
+    <t>PaymentType</t>
+  </si>
+  <si>
+    <t>CASH</t>
+  </si>
+  <si>
+    <t>selectCounter</t>
+  </si>
+  <si>
+    <t>Cornea</t>
+  </si>
+  <si>
+    <t>Foreign country</t>
+  </si>
+  <si>
+    <t>AFRICA</t>
+  </si>
+  <si>
+    <t>zip code</t>
+  </si>
+  <si>
+    <t>5464</t>
+  </si>
+  <si>
+    <t>5465</t>
+  </si>
+  <si>
+    <t>MRN</t>
+  </si>
+  <si>
+    <t>P6089-658</t>
+  </si>
+  <si>
+    <t>P6089-659</t>
+  </si>
+  <si>
+    <t>UIN</t>
+  </si>
+  <si>
+    <t>0024427536</t>
+  </si>
+  <si>
+    <t>0024427537</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>UNIT-3</t>
+  </si>
+  <si>
+    <t>UNIT-4</t>
+  </si>
+  <si>
+    <t>FREE</t>
+  </si>
+  <si>
+    <t>CAMP</t>
+  </si>
+  <si>
+    <t>FFFF</t>
+  </si>
+  <si>
+    <t>CCCC</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>25-06-2002</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>S/O</t>
+  </si>
+  <si>
+    <t>iii</t>
+  </si>
+  <si>
+    <t>Referral</t>
+  </si>
+  <si>
+    <t>12565</t>
+  </si>
+  <si>
+    <t>20-06-2028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIT-3 </t>
+  </si>
+  <si>
     <t>Indian</t>
   </si>
   <si>
-    <t>DoorStreet</t>
-  </si>
-  <si>
-    <t>98 rrr street</t>
-  </si>
-  <si>
-    <t>locality</t>
-  </si>
-  <si>
-    <t>inside madurai</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>madurai</t>
-  </si>
-  <si>
-    <t>Area</t>
-  </si>
-  <si>
-    <t>BEE BEE KULAM</t>
-  </si>
-  <si>
-    <t>PinCode</t>
-  </si>
-  <si>
-    <t>Taluk</t>
-  </si>
-  <si>
-    <t>MADURAI - GENL</t>
-  </si>
-  <si>
-    <t>MobileNo</t>
-  </si>
-  <si>
-    <t>8456219575</t>
-  </si>
-  <si>
-    <t>Email</t>
+    <t>100 rrr street</t>
+  </si>
+  <si>
+    <t>7851200369</t>
+  </si>
+  <si>
+    <t>emailihms02@gmail.com</t>
   </si>
   <si>
     <t>emailihms48@gmail.com</t>
   </si>
   <si>
-    <t>PurposeVisit</t>
-  </si>
-  <si>
-    <t>Review</t>
-  </si>
-  <si>
-    <t>ConsentForm</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Assign doctor</t>
-  </si>
-  <si>
-    <t>Esha</t>
-  </si>
-  <si>
-    <t>PatientSubCategory</t>
+    <t>Subsidy</t>
   </si>
   <si>
     <t>Concession</t>
   </si>
   <si>
-    <t>SubsidyApprovedBy</t>
-  </si>
-  <si>
-    <t>AEH-DINDIGUL</t>
-  </si>
-  <si>
-    <t>Subsidy granted</t>
-  </si>
-  <si>
-    <t>Subsidy Reason</t>
-  </si>
-  <si>
-    <t>CAMP SUBSIDY</t>
-  </si>
-  <si>
-    <t>Subsidy remarks</t>
-  </si>
-  <si>
-    <t>Subsidy remarks are entered</t>
-  </si>
-  <si>
-    <t>ConcessionApprovedBy</t>
-  </si>
-  <si>
-    <t>Concession granted</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>Concession Reason</t>
-  </si>
-  <si>
-    <t>Concession remarks</t>
-  </si>
-  <si>
-    <t>Concession remarks are entered</t>
-  </si>
-  <si>
-    <t>Patient category</t>
-  </si>
-  <si>
-    <t>FULL PAYMENT</t>
+    <t>32</t>
   </si>
   <si>
     <t>CORPORATE</t>
   </si>
   <si>
-    <t>Corporate name</t>
-  </si>
-  <si>
-    <t>NIND STUDY</t>
-  </si>
-  <si>
-    <t>Document Ref.no</t>
-  </si>
-  <si>
-    <t>458967</t>
-  </si>
-  <si>
-    <t>Employee grade</t>
-  </si>
-  <si>
-    <t>EMPLOYEE</t>
-  </si>
-  <si>
-    <t>Employee code</t>
-  </si>
-  <si>
-    <t>1526349</t>
-  </si>
-  <si>
-    <t>Claim id</t>
-  </si>
-  <si>
-    <t>1452</t>
-  </si>
-  <si>
-    <t>Corporate remarks</t>
-  </si>
-  <si>
-    <t>Corporate remarks is entered</t>
-  </si>
-  <si>
-    <t>PaymentType</t>
-  </si>
-  <si>
-    <t>CASH</t>
-  </si>
-  <si>
-    <t>selectCounter</t>
-  </si>
-  <si>
-    <t>Cornea</t>
-  </si>
-  <si>
-    <t>Foreign country</t>
-  </si>
-  <si>
-    <t>AFRICA</t>
-  </si>
-  <si>
-    <t>zip code</t>
-  </si>
-  <si>
-    <t>5464</t>
-  </si>
-  <si>
-    <t>MRN</t>
-  </si>
-  <si>
-    <t>P6089-619</t>
-  </si>
-  <si>
-    <t>P6089-620</t>
-  </si>
-  <si>
-    <t>UIN</t>
-  </si>
-  <si>
-    <t>0024427485</t>
-  </si>
-  <si>
-    <t>0024427487</t>
-  </si>
-  <si>
-    <t>Location</t>
-  </si>
-  <si>
-    <t>UNIT-3</t>
-  </si>
-  <si>
-    <t>FREE</t>
-  </si>
-  <si>
-    <t>CAMP</t>
-  </si>
-  <si>
-    <t>FFFF</t>
-  </si>
-  <si>
-    <t>CCCC</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>25-06-2002</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>S/O</t>
-  </si>
-  <si>
-    <t>iii</t>
-  </si>
-  <si>
-    <t>Referral</t>
-  </si>
-  <si>
-    <t>12564</t>
-  </si>
-  <si>
-    <t>12565</t>
-  </si>
-  <si>
-    <t>20-06-2027</t>
-  </si>
-  <si>
-    <t>20-06-2028</t>
-  </si>
-  <si>
-    <t>07-07-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIT-2 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIT-3 </t>
-  </si>
-  <si>
-    <t>99 rrr street</t>
-  </si>
-  <si>
-    <t>100 rrr street</t>
-  </si>
-  <si>
-    <t>7851200369</t>
-  </si>
-  <si>
-    <t>emailihms02@gmail.com</t>
-  </si>
-  <si>
-    <t>Subsidy</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>458968</t>
-  </si>
-  <si>
     <t>458969</t>
   </si>
   <si>
-    <t>1523445</t>
-  </si>
-  <si>
     <t>4573239</t>
   </si>
   <si>
-    <t>3048342</t>
-  </si>
-  <si>
     <t>6098136</t>
   </si>
   <si>
     <t>HOSPITAL ACCOUNT</t>
   </si>
   <si>
-    <t>Orbit</t>
-  </si>
-  <si>
     <t>F2680-543</t>
   </si>
   <si>
     <t>C-150</t>
   </si>
   <si>
-    <t>P6089-442</t>
-  </si>
-  <si>
     <t>0024427262</t>
   </si>
   <si>
     <t>0024427486</t>
   </si>
   <si>
-    <t>0024427271</t>
-  </si>
-  <si>
     <t>CAMP UNIT</t>
   </si>
   <si>
     <t>Total Collection Registration</t>
   </si>
   <si>
-    <t>₹ 2100</t>
+    <t>₹ 0</t>
   </si>
   <si>
     <t>Unit Load Registration</t>
@@ -482,12 +482,15 @@
     <t>dateReprint</t>
   </si>
   <si>
-    <t>23-07-2026</t>
+    <t>24-07-2026</t>
   </si>
   <si>
     <t>uinReprint</t>
   </si>
   <si>
+    <t>0024427546</t>
+  </si>
+  <si>
     <t>ReprintChoice</t>
   </si>
   <si>
@@ -497,36 +500,56 @@
     <t>ReceiptReprint</t>
   </si>
   <si>
-    <t>O26271958 - 23/07/2026</t>
+    <t>O26272018 - 24/07/2026</t>
   </si>
   <si>
     <t>uinRouteCard</t>
   </si>
   <si>
-    <t>0024427439</t>
+    <t>common uin</t>
+  </si>
+  <si>
+    <t>edit mobile number</t>
+  </si>
+  <si>
+    <t>9562148759</t>
+  </si>
+  <si>
+    <t>PATIENT ENQUIRY VALIDATION</t>
+  </si>
+  <si>
+    <t>Enquiry patient type</t>
+  </si>
+  <si>
+    <t>IP</t>
   </si>
   <si>
     <t>uinBilling</t>
   </si>
   <si>
-    <t>P6089-658</t>
-  </si>
-  <si>
-    <t>0024427536</t>
-  </si>
-  <si>
-    <t>P6089-659</t>
-  </si>
-  <si>
-    <t>0024427537</t>
+    <t>pin number</t>
+  </si>
+  <si>
+    <t>668</t>
+  </si>
+  <si>
+    <t>test name</t>
+  </si>
+  <si>
+    <t>ACE TEST</t>
+  </si>
+  <si>
+    <t>test location</t>
+  </si>
+  <si>
+    <t>BARRAGE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -545,8 +568,15 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -563,6 +593,11 @@
         <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -572,11 +607,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -877,14 +914,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="39.28516"/>
-    <col min="2" max="2" customWidth="true" width="40.28516"/>
-    <col min="3" max="3" customWidth="true" width="28.71094"/>
-    <col min="4" max="4" customWidth="true" width="28.71094"/>
-    <col min="5" max="5" customWidth="true" width="28.71094"/>
+    <col min="1" max="1" width="39.28516" customWidth="1"/>
+    <col min="2" max="2" width="40.28516" customWidth="1"/>
+    <col min="3" max="3" width="28.71094" customWidth="1"/>
+    <col min="4" max="4" width="28.71094" customWidth="1"/>
+    <col min="5" max="5" width="28.71094" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -899,7 +935,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -910,7 +946,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -921,7 +957,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -932,217 +968,217 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="2">
-        <v>25</v>
+      <c r="C5" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>10</v>
+      <c r="A6" t="s">
+        <v>11</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="0">
-        <v>13</v>
+      <c r="A7" t="s">
+        <v>14</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="s" s="0">
-        <v>15</v>
+      <c r="A8" t="s">
+        <v>16</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="s" s="0">
-        <v>17</v>
+      <c r="A9" t="s">
+        <v>18</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="s" s="0">
-        <v>21</v>
+      <c r="A11" t="s">
+        <v>22</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="s" s="0">
-        <v>23</v>
+      <c r="A12" t="s">
+        <v>25</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="s" s="0">
-        <v>25</v>
+      <c r="A13" t="s">
+        <v>28</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="s" s="0">
-        <v>27</v>
+      <c r="A14" t="s">
+        <v>30</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="s" s="0">
-        <v>29</v>
+      <c r="A15" t="s">
+        <v>33</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="B16" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="C16" t="s" s="0">
-        <v>32</v>
+      <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="s" s="0">
-        <v>33</v>
-      </c>
-      <c r="B17" t="s" s="0">
-        <v>34</v>
-      </c>
-      <c r="C17" t="s" s="0">
-        <v>34</v>
+      <c r="A17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="s" s="0">
-        <v>35</v>
-      </c>
-      <c r="B18" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="C18" t="s" s="0">
-        <v>36</v>
+      <c r="A18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="s" s="0">
-        <v>37</v>
+      <c r="A19" t="s">
+        <v>41</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="s" s="0">
-        <v>40</v>
+      <c r="A20" t="s">
+        <v>43</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="s" s="0">
-        <v>42</v>
+      <c r="A21" t="s">
+        <v>46</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="s" s="0">
-        <v>44</v>
+      <c r="A22" t="s">
+        <v>48</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="s" s="0">
-        <v>46</v>
+      <c r="A23" t="s">
+        <v>50</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="s" s="0">
-        <v>48</v>
+      <c r="A24" t="s">
+        <v>52</v>
       </c>
       <c r="B24" s="2">
         <v>645126</v>
@@ -1152,94 +1188,92 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="s" s="0">
-        <v>49</v>
+      <c r="A25" t="s">
+        <v>53</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="s" s="0">
-        <v>51</v>
+      <c r="A26" t="s">
+        <v>55</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C26" s="2">
-        <v>8457962513</v>
+        <v>56</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="s" s="0">
-        <v>53</v>
+      <c r="A27" t="s">
+        <v>57</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="s" s="0">
-        <v>55</v>
+      <c r="A28" t="s">
+        <v>59</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="s" s="0">
-        <v>57</v>
+      <c r="A29" t="s">
+        <v>61</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="s" s="0">
-        <v>59</v>
+      <c r="A30" t="s">
+        <v>63</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B31" s="2"/>
-      <c r="C31" s="2" t="s">
-        <v>62</v>
-      </c>
+      <c r="C31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" t="s" s="0">
-        <v>63</v>
+      <c r="A32" t="s">
+        <v>66</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="s" s="0">
-        <v>65</v>
+      <c r="A33" t="s">
+        <v>68</v>
       </c>
       <c r="B33" s="2">
         <v>50</v>
@@ -1249,217 +1283,223 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="s" s="0">
-        <v>66</v>
+      <c r="A34" t="s">
+        <v>69</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>71</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>73</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="s" s="0">
-        <v>68</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="s" s="0">
+    <row r="37">
+      <c r="A37" t="s">
+        <v>74</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>77</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="s" s="0">
-        <v>71</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="s" s="0">
-        <v>73</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="C38" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="s" s="0">
-        <v>74</v>
+      <c r="A39" t="s">
+        <v>78</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="s" s="0">
-        <v>79</v>
+      <c r="A41" t="s">
+        <v>82</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="s" s="0">
-        <v>81</v>
+      <c r="A42" t="s">
+        <v>84</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="s" s="0">
-        <v>83</v>
+      <c r="A43" t="s">
+        <v>87</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="s" s="0">
-        <v>85</v>
+      <c r="A44" t="s">
+        <v>89</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="s" s="0">
-        <v>87</v>
+      <c r="A45" t="s">
+        <v>92</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="s" s="0">
-        <v>89</v>
+      <c r="A46" t="s">
+        <v>95</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="B47" t="s" s="0">
-        <v>92</v>
-      </c>
-      <c r="C47" t="s" s="0">
-        <v>92</v>
+        <v>97</v>
+      </c>
+      <c r="B47" t="s">
+        <v>98</v>
+      </c>
+      <c r="C47" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="s" s="0">
-        <v>93</v>
-      </c>
-      <c r="B48" t="s" s="0">
-        <v>94</v>
-      </c>
-      <c r="C48" t="s" s="0">
-        <v>94</v>
+      <c r="A48" t="s">
+        <v>99</v>
+      </c>
+      <c r="B48" t="s">
+        <v>100</v>
+      </c>
+      <c r="C48" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="B49" t="s" s="0">
-        <v>96</v>
+      <c r="A49" t="s">
+        <v>101</v>
+      </c>
+      <c r="B49" t="s">
+        <v>102</v>
+      </c>
+      <c r="C49" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="s" s="0">
-        <v>97</v>
+      <c r="A50" t="s">
+        <v>103</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>98</v>
+        <v>104</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="s" s="0">
-        <v>99</v>
-      </c>
-      <c r="B58" t="s" s="0">
-        <v>162</v>
-      </c>
-      <c r="C58" t="s" s="0">
-        <v>164</v>
+      <c r="A58" t="s">
+        <v>106</v>
+      </c>
+      <c r="B58" t="s">
+        <v>107</v>
+      </c>
+      <c r="C58" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="s" s="0">
-        <v>102</v>
+      <c r="A59" t="s">
+        <v>109</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="C59" t="s" s="0">
-        <v>165</v>
+        <v>110</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="s" s="0">
-        <v>105</v>
+      <c r="A60" t="s">
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="61">
@@ -1471,21 +1511,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="29.71094"/>
-    <col min="2" max="2" customWidth="true" width="31.42578"/>
-    <col min="3" max="3" customWidth="true" width="34.0"/>
-    <col min="4" max="4" customWidth="true" width="37.42578"/>
+    <col min="1" max="1" width="29.71094" customWidth="1"/>
+    <col min="2" max="2" width="31.42578" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="37.42578" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -1510,10 +1549,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>5</v>
@@ -1532,265 +1571,275 @@
       <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2">
         <v>25</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="C5" s="2">
         <v>25</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>9</v>
+      <c r="D5" s="2">
+        <v>25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>113</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>114</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>117</v>
+        <v>24</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>119</v>
+        <v>27</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>121</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>122</v>
+        <v>32</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="B16" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="C16" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="D16" t="s" s="0">
-        <v>32</v>
+      <c r="A16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="s" s="0">
-        <v>34</v>
-      </c>
-      <c r="B17" t="s" s="0">
-        <v>34</v>
-      </c>
-      <c r="C17" t="s" s="0">
-        <v>34</v>
-      </c>
-      <c r="D17" t="s" s="0">
-        <v>34</v>
+      <c r="A17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="B18" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="C18" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="D18" t="s" s="0">
-        <v>36</v>
+      <c r="A18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>39</v>
+        <v>128</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>39</v>
+        <v>128</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>39</v>
+        <v>128</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>39</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>124</v>
+        <v>45</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="2"/>
+        <v>44</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D21" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D22" s="2"/>
+        <v>49</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D23" s="2"/>
+        <v>51</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2">
@@ -1802,25 +1851,27 @@
       <c r="C24" s="2">
         <v>645126</v>
       </c>
-      <c r="D24" s="2"/>
+      <c r="D24" s="2">
+        <v>645126</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B26" s="2">
         <v>8457962513</v>
@@ -1828,87 +1879,93 @@
       <c r="C26" s="2">
         <v>8457962513</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>52</v>
+      <c r="D26" s="2">
+        <v>8457962513</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>54</v>
+        <v>132</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D27" s="2"/>
+        <v>132</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D31" s="2"/>
+        <v>134</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D32" s="2"/>
+        <v>67</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2">
@@ -1920,234 +1977,257 @@
       <c r="C33" s="2">
         <v>50</v>
       </c>
-      <c r="D33" s="2"/>
+      <c r="D33" s="2">
+        <v>50</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D34" s="2"/>
+        <v>70</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D35" s="2"/>
+        <v>72</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D36" s="2"/>
+        <v>67</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>129</v>
+        <v>76</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D37" s="2"/>
+        <v>75</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D38" s="2"/>
+        <v>70</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D39" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>78</v>
+        <v>136</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>78</v>
+        <v>136</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>77</v>
+        <v>136</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="s">
-        <v>131</v>
+        <v>86</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="s">
-        <v>133</v>
+        <v>91</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="s">
-        <v>135</v>
+        <v>94</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="s" s="0">
-        <v>137</v>
-      </c>
-      <c r="B47" t="s" s="0">
-        <v>137</v>
-      </c>
-      <c r="C47" t="s" s="0">
-        <v>92</v>
-      </c>
-      <c r="D47" t="s" s="0">
-        <v>92</v>
+      <c r="A47" t="s">
+        <v>140</v>
+      </c>
+      <c r="B47" t="s">
+        <v>140</v>
+      </c>
+      <c r="C47" t="s">
+        <v>98</v>
+      </c>
+      <c r="D47" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="48">
-      <c r="C48" t="s" s="0">
-        <v>94</v>
-      </c>
-      <c r="D48" t="s" s="0">
-        <v>138</v>
+      <c r="C48" t="s">
+        <v>100</v>
+      </c>
+      <c r="D48" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="52">
-      <c r="D52" s="2"/>
+      <c r="D52"/>
     </row>
     <row r="55">
-      <c r="A55" t="s" s="0">
-        <v>139</v>
-      </c>
-      <c r="B55" t="s" s="0">
-        <v>140</v>
-      </c>
-      <c r="D55" t="s" s="0">
+      <c r="A55" t="s">
         <v>141</v>
       </c>
+      <c r="B55" t="s">
+        <v>142</v>
+      </c>
+      <c r="D55"/>
     </row>
     <row r="56">
-      <c r="A56" t="s" s="0">
-        <v>142</v>
-      </c>
-      <c r="B56" t="s" s="0">
+      <c r="A56" t="s">
         <v>143</v>
       </c>
-      <c r="D56" s="2" t="s">
+      <c r="B56" t="s">
         <v>144</v>
       </c>
+      <c r="D56"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B57" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="B57" t="s">
         <v>145</v>
       </c>
-      <c r="D57" s="2" t="s">
-        <v>106</v>
+      <c r="D57"/>
+    </row>
+    <row r="58">
+      <c r="D58" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="D59" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="D60" s="2" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -2156,84 +2236,204 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="33.0"/>
-    <col min="2" max="2" customWidth="true" width="111.5703"/>
-    <col min="3" max="3" customWidth="true" width="20.28516"/>
+    <col min="1" max="1" width="38.71094" customWidth="1"/>
+    <col min="2" max="2" width="111.5703" customWidth="1"/>
+    <col min="3" max="3" width="20.28516" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>146</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" s="2" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>148</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" s="2" t="s">
         <v>149</v>
       </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
         <v>150</v>
       </c>
+      <c r="B5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>151</v>
       </c>
-      <c r="B6" t="s" s="0">
-        <v>56</v>
+      <c r="B6" s="2" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>152</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="B7" s="2" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="s" s="0">
+      <c r="A8" t="s">
         <v>154</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>103</v>
+        <v>155</v>
       </c>
       <c r="C8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" t="s" s="0">
+      <c r="A9" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>158</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>160</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="B9" t="s" s="0">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="0">
-        <v>157</v>
-      </c>
-      <c r="B10" t="s" s="0">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="0">
-        <v>159</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>160</v>
-      </c>
       <c r="C11" s="2"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>162</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="2"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="4"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B16" s="2"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>165</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="2"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="2"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="2"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="2"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="2"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="2"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="2"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="2"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="2"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="2"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="2"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="2"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="2"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="2"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="2"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="2"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="2"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="2"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="2"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="2"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="2"/>
+    </row>
+    <row r="40">
+      <c r="B40" s="2"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="2"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="2"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="2"/>
     </row>
   </sheetData>
 </worksheet>
@@ -2241,20 +2441,43 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="2" width="25.42578"/>
-    <col min="2" max="2" customWidth="true" style="2" width="23.42578"/>
-    <col min="3" max="16384" style="2" width="9.140625"/>
+    <col min="1" max="1" width="25.42578" style="2" customWidth="1"/>
+    <col min="2" max="2" width="23.42578" style="2" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>160</v>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>